<commit_message>
Add scripts for grading metrics and element distribution analysis
- Implemented `aggregate_combined_grading_metrics.py` to aggregate grading metrics from human and LLM auto-grading sheets, producing a consolidated CSV output.
- Created `compute_element_distribution.py` to compute the distribution of state machine elements across various systems, generating a CSV file with counts of different element types.
- Developed `compute_raw_grading_counts.py` to directly compute grading counts (N, TP, FP, FN) from raw data sheets, addressing issues with previous metrics calculations and ensuring accurate results.
- Updated `Distribution_of_State_Machine_Elements_Across_Systems.csv` with corrected totals based on new calculations.
</commit_message>
<xml_diff>
--- a/Digital Chess Clock/Grading/1 stage/3-examples/Digital-Chess-Clock_Grading_1-stage_2026-02-28_3-examples_CombinedHumanGradingVsClaude4.5SonnetAutoGrading_Claude4.5SonnetGeneration.xlsx
+++ b/Digital Chess Clock/Grading/1 stage/3-examples/Digital-Chess-Clock_Grading_1-stage_2026-02-28_3-examples_CombinedHumanGradingVsClaude4.5SonnetAutoGrading_Claude4.5SonnetGeneration.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marc-antoinenadeau/Desktop/Evaluations 2/Digital Chess Clock/Grading/1 stage/2026-02-28/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marc-antoinenadeau/Desktop/B.Eng Software Engineering /7th Semester/Capstone/Code/Evaluations/Digital Chess Clock/Grading/1 stage/3-examples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{500E1254-69F7-584D-A147-415F9543E40C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC7A341F-59BC-154D-BE50-801A50031B7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17480" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17300" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Chess Clock" sheetId="1" r:id="rId1"/>
@@ -1136,19 +1136,19 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -15692,16 +15692,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="76" t="s">
+      <c r="A1" s="79" t="s">
         <v>114</v>
       </c>
-      <c r="B1" s="77"/>
-      <c r="C1" s="77"/>
-      <c r="D1" s="77"/>
-      <c r="E1" s="77"/>
-      <c r="F1" s="77"/>
-      <c r="G1" s="77"/>
-      <c r="H1" s="77"/>
+      <c r="B1" s="80"/>
+      <c r="C1" s="80"/>
+      <c r="D1" s="80"/>
+      <c r="E1" s="80"/>
+      <c r="F1" s="80"/>
+      <c r="G1" s="80"/>
+      <c r="H1" s="80"/>
       <c r="J1" s="28" t="s">
         <v>115</v>
       </c>
@@ -16008,16 +16008,16 @@
     </row>
     <row r="11" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="12" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A12" s="76" t="s">
+      <c r="A12" s="79" t="s">
         <v>127</v>
       </c>
-      <c r="B12" s="77"/>
-      <c r="C12" s="77"/>
-      <c r="D12" s="77"/>
-      <c r="E12" s="77"/>
-      <c r="F12" s="77"/>
-      <c r="G12" s="77"/>
-      <c r="H12" s="77"/>
+      <c r="B12" s="80"/>
+      <c r="C12" s="80"/>
+      <c r="D12" s="80"/>
+      <c r="E12" s="80"/>
+      <c r="F12" s="80"/>
+      <c r="G12" s="80"/>
+      <c r="H12" s="80"/>
     </row>
     <row r="13" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="29" t="s">
@@ -16050,7 +16050,7 @@
         <v>128</v>
       </c>
       <c r="B14" s="32">
-        <f>COUNTIF('Chess Clock'!$A$2:$A$44, A14)</f>
+        <f>COUNTIF('Chess Clock'!$A$2:$A$46, A14)</f>
         <v>3</v>
       </c>
       <c r="C14" s="33">
@@ -16083,8 +16083,8 @@
         <v>2</v>
       </c>
       <c r="B15" s="32">
-        <f>COUNTIF('Chess Clock'!$A$2:$A$44, A15)</f>
-        <v>12</v>
+        <f>COUNTIF('Chess Clock'!$A$2:$A$46, A15)</f>
+        <v>13</v>
       </c>
       <c r="C15" s="33">
         <f>SUMIF('LLM Grading'!$A$2:$A$46, $A15, 'LLM Grading'!$C$2:$C$46)</f>
@@ -16104,11 +16104,11 @@
       </c>
       <c r="G15" s="33">
         <f t="shared" si="6"/>
-        <v>0.625</v>
+        <v>0.57692307692307687</v>
       </c>
       <c r="H15" s="33">
         <f t="shared" si="7"/>
-        <v>0.73170731707317083</v>
+        <v>0.69767441860465118</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -16116,8 +16116,8 @@
         <v>4</v>
       </c>
       <c r="B16" s="32">
-        <f>COUNTIF('Chess Clock'!$A$2:$A$44, A16)</f>
-        <v>13</v>
+        <f>COUNTIF('Chess Clock'!$A$2:$A$46, A16)</f>
+        <v>14</v>
       </c>
       <c r="C16" s="33">
         <f>SUMIF('LLM Grading'!$A$2:$A$46, $A16, 'LLM Grading'!$C$2:$C$46)</f>
@@ -16137,11 +16137,11 @@
       </c>
       <c r="G16" s="33">
         <f t="shared" si="6"/>
-        <v>0.69230769230769229</v>
+        <v>0.6428571428571429</v>
       </c>
       <c r="H16" s="33">
         <f t="shared" si="7"/>
-        <v>0.81818181818181812</v>
+        <v>0.78260869565217395</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -16215,7 +16215,7 @@
         <v>31</v>
       </c>
       <c r="B19" s="32">
-        <f>COUNTIF('Chess Clock'!$A$2:$A$44, A19)</f>
+        <f>COUNTIF('Chess Clock'!$A$2:$A$46, A19)</f>
         <v>1</v>
       </c>
       <c r="C19" s="33">
@@ -16282,7 +16282,7 @@
       </c>
       <c r="B21" s="33">
         <f t="shared" ref="B21:E21" si="8">SUM(B14:B20)</f>
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C21" s="33">
         <f t="shared" si="8"/>
@@ -16302,11 +16302,11 @@
       </c>
       <c r="G21" s="33">
         <f t="shared" si="6"/>
-        <v>0.46511627906976744</v>
+        <v>0.44444444444444442</v>
       </c>
       <c r="H21" s="33">
         <f t="shared" si="7"/>
-        <v>0.61538461538461531</v>
+        <v>0.59701492537313428</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -17330,24 +17330,24 @@
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="82" t="s">
+      <c r="C1" s="76" t="s">
         <v>165</v>
       </c>
-      <c r="D1" s="82" t="s">
+      <c r="D1" s="76" t="s">
         <v>64</v>
       </c>
       <c r="E1" s="36"/>
-      <c r="F1" s="78" t="s">
+      <c r="F1" s="77" t="s">
         <v>129</v>
       </c>
-      <c r="G1" s="79"/>
-      <c r="H1" s="79"/>
-      <c r="I1" s="79"/>
-      <c r="L1" s="80" t="s">
+      <c r="G1" s="78"/>
+      <c r="H1" s="78"/>
+      <c r="I1" s="78"/>
+      <c r="L1" s="81" t="s">
         <v>130</v>
       </c>
-      <c r="M1" s="81"/>
-      <c r="N1" s="81"/>
+      <c r="M1" s="82"/>
+      <c r="N1" s="82"/>
     </row>
     <row r="2" spans="1:14" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="str">
@@ -17617,17 +17617,17 @@
         <v>0.5</v>
       </c>
       <c r="E8" s="36"/>
-      <c r="F8" s="78" t="s">
+      <c r="F8" s="77" t="s">
         <v>145</v>
       </c>
-      <c r="G8" s="79"/>
-      <c r="H8" s="79"/>
-      <c r="I8" s="79"/>
-      <c r="L8" s="80" t="s">
+      <c r="G8" s="78"/>
+      <c r="H8" s="78"/>
+      <c r="I8" s="78"/>
+      <c r="L8" s="81" t="s">
         <v>146</v>
       </c>
-      <c r="M8" s="81"/>
-      <c r="N8" s="81"/>
+      <c r="M8" s="82"/>
+      <c r="N8" s="82"/>
     </row>
     <row r="9" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="4" t="str">
@@ -17894,17 +17894,17 @@
         <v>1</v>
       </c>
       <c r="E15" s="36"/>
-      <c r="F15" s="78" t="s">
+      <c r="F15" s="77" t="s">
         <v>147</v>
       </c>
-      <c r="G15" s="79"/>
-      <c r="H15" s="79"/>
-      <c r="I15" s="79"/>
-      <c r="L15" s="80" t="s">
+      <c r="G15" s="78"/>
+      <c r="H15" s="78"/>
+      <c r="I15" s="78"/>
+      <c r="L15" s="81" t="s">
         <v>148</v>
       </c>
-      <c r="M15" s="81"/>
-      <c r="N15" s="81"/>
+      <c r="M15" s="82"/>
+      <c r="N15" s="82"/>
     </row>
     <row r="16" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="4" t="str">
@@ -18171,17 +18171,17 @@
         <v>0.5</v>
       </c>
       <c r="E22" s="36"/>
-      <c r="F22" s="78" t="s">
+      <c r="F22" s="77" t="s">
         <v>149</v>
       </c>
-      <c r="G22" s="79"/>
-      <c r="H22" s="79"/>
-      <c r="I22" s="79"/>
-      <c r="L22" s="80" t="s">
+      <c r="G22" s="78"/>
+      <c r="H22" s="78"/>
+      <c r="I22" s="78"/>
+      <c r="L22" s="81" t="s">
         <v>150</v>
       </c>
-      <c r="M22" s="81"/>
-      <c r="N22" s="81"/>
+      <c r="M22" s="82"/>
+      <c r="N22" s="82"/>
     </row>
     <row r="23" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="4" t="str">
@@ -18448,17 +18448,17 @@
         <v>0</v>
       </c>
       <c r="E29" s="36"/>
-      <c r="F29" s="78" t="s">
+      <c r="F29" s="77" t="s">
         <v>151</v>
       </c>
-      <c r="G29" s="79"/>
-      <c r="H29" s="79"/>
-      <c r="I29" s="79"/>
-      <c r="L29" s="80" t="s">
+      <c r="G29" s="78"/>
+      <c r="H29" s="78"/>
+      <c r="I29" s="78"/>
+      <c r="L29" s="81" t="s">
         <v>152</v>
       </c>
-      <c r="M29" s="81"/>
-      <c r="N29" s="81"/>
+      <c r="M29" s="82"/>
+      <c r="N29" s="82"/>
     </row>
     <row r="30" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A30" s="4" t="str">
@@ -18725,17 +18725,17 @@
         <v>0</v>
       </c>
       <c r="E36" s="36"/>
-      <c r="F36" s="78" t="s">
+      <c r="F36" s="77" t="s">
         <v>153</v>
       </c>
-      <c r="G36" s="79"/>
-      <c r="H36" s="79"/>
-      <c r="I36" s="79"/>
-      <c r="L36" s="80" t="s">
+      <c r="G36" s="78"/>
+      <c r="H36" s="78"/>
+      <c r="I36" s="78"/>
+      <c r="L36" s="81" t="s">
         <v>154</v>
       </c>
-      <c r="M36" s="81"/>
-      <c r="N36" s="81"/>
+      <c r="M36" s="82"/>
+      <c r="N36" s="82"/>
     </row>
     <row r="37" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A37" s="4" t="str">
@@ -19002,17 +19002,17 @@
         <v>1</v>
       </c>
       <c r="E43" s="36"/>
-      <c r="F43" s="78" t="s">
+      <c r="F43" s="77" t="s">
         <v>155</v>
       </c>
-      <c r="G43" s="79"/>
-      <c r="H43" s="79"/>
-      <c r="I43" s="79"/>
-      <c r="L43" s="80" t="s">
+      <c r="G43" s="78"/>
+      <c r="H43" s="78"/>
+      <c r="I43" s="78"/>
+      <c r="L43" s="81" t="s">
         <v>156</v>
       </c>
-      <c r="M43" s="81"/>
-      <c r="N43" s="81"/>
+      <c r="M43" s="82"/>
+      <c r="N43" s="82"/>
     </row>
     <row r="44" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A44" s="4" t="str">
@@ -19279,17 +19279,17 @@
         <v>1</v>
       </c>
       <c r="E50" s="36"/>
-      <c r="F50" s="78" t="s">
+      <c r="F50" s="77" t="s">
         <v>157</v>
       </c>
-      <c r="G50" s="79"/>
-      <c r="H50" s="79"/>
-      <c r="I50" s="79"/>
-      <c r="L50" s="80" t="s">
+      <c r="G50" s="78"/>
+      <c r="H50" s="78"/>
+      <c r="I50" s="78"/>
+      <c r="L50" s="81" t="s">
         <v>158</v>
       </c>
-      <c r="M50" s="81"/>
-      <c r="N50" s="81"/>
+      <c r="M50" s="82"/>
+      <c r="N50" s="82"/>
     </row>
     <row r="51" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A51" s="4" t="str">
@@ -20541,6 +20541,12 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="F1:I1"/>
+    <mergeCell ref="L1:N1"/>
+    <mergeCell ref="F8:I8"/>
+    <mergeCell ref="L8:N8"/>
+    <mergeCell ref="F15:I15"/>
+    <mergeCell ref="L15:N15"/>
     <mergeCell ref="L22:N22"/>
     <mergeCell ref="F50:I50"/>
     <mergeCell ref="L50:N50"/>
@@ -20551,12 +20557,6 @@
     <mergeCell ref="L36:N36"/>
     <mergeCell ref="F43:I43"/>
     <mergeCell ref="L43:N43"/>
-    <mergeCell ref="F1:I1"/>
-    <mergeCell ref="L1:N1"/>
-    <mergeCell ref="F8:I8"/>
-    <mergeCell ref="L8:N8"/>
-    <mergeCell ref="F15:I15"/>
-    <mergeCell ref="L15:N15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
@@ -20598,25 +20598,25 @@
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="82" t="s">
+      <c r="C1" s="76" t="s">
         <v>165</v>
       </c>
-      <c r="D1" s="82" t="s">
+      <c r="D1" s="76" t="s">
         <v>64</v>
       </c>
       <c r="E1" s="36"/>
-      <c r="F1" s="78" t="s">
+      <c r="F1" s="77" t="s">
         <v>129</v>
       </c>
-      <c r="G1" s="79"/>
-      <c r="H1" s="79"/>
-      <c r="I1" s="79"/>
-      <c r="L1" s="78" t="s">
+      <c r="G1" s="78"/>
+      <c r="H1" s="78"/>
+      <c r="I1" s="78"/>
+      <c r="L1" s="77" t="s">
         <v>159</v>
       </c>
-      <c r="M1" s="79"/>
-      <c r="N1" s="79"/>
-      <c r="O1" s="79"/>
+      <c r="M1" s="78"/>
+      <c r="N1" s="78"/>
+      <c r="O1" s="78"/>
     </row>
     <row r="2" spans="1:24" ht="15.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="str">
@@ -21020,12 +21020,12 @@
         <v>0.5</v>
       </c>
       <c r="E8" s="36"/>
-      <c r="F8" s="78" t="s">
+      <c r="F8" s="77" t="s">
         <v>145</v>
       </c>
-      <c r="G8" s="79"/>
-      <c r="H8" s="79"/>
-      <c r="I8" s="79"/>
+      <c r="G8" s="78"/>
+      <c r="H8" s="78"/>
+      <c r="I8" s="78"/>
     </row>
     <row r="9" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="4" t="str">
@@ -21415,12 +21415,12 @@
         <v>1</v>
       </c>
       <c r="E15" s="36"/>
-      <c r="F15" s="78" t="s">
+      <c r="F15" s="77" t="s">
         <v>147</v>
       </c>
-      <c r="G15" s="79"/>
-      <c r="H15" s="79"/>
-      <c r="I15" s="79"/>
+      <c r="G15" s="78"/>
+      <c r="H15" s="78"/>
+      <c r="I15" s="78"/>
     </row>
     <row r="16" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="4" t="str">
@@ -21810,12 +21810,12 @@
         <v>0.5</v>
       </c>
       <c r="E22" s="36"/>
-      <c r="F22" s="78" t="s">
+      <c r="F22" s="77" t="s">
         <v>149</v>
       </c>
-      <c r="G22" s="79"/>
-      <c r="H22" s="79"/>
-      <c r="I22" s="79"/>
+      <c r="G22" s="78"/>
+      <c r="H22" s="78"/>
+      <c r="I22" s="78"/>
     </row>
     <row r="23" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="4" t="str">
@@ -22205,12 +22205,12 @@
         <v>0</v>
       </c>
       <c r="E29" s="36"/>
-      <c r="F29" s="78" t="s">
+      <c r="F29" s="77" t="s">
         <v>151</v>
       </c>
-      <c r="G29" s="79"/>
-      <c r="H29" s="79"/>
-      <c r="I29" s="79"/>
+      <c r="G29" s="78"/>
+      <c r="H29" s="78"/>
+      <c r="I29" s="78"/>
     </row>
     <row r="30" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A30" s="4" t="str">
@@ -22600,12 +22600,12 @@
         <v>0</v>
       </c>
       <c r="E36" s="36"/>
-      <c r="F36" s="78" t="s">
+      <c r="F36" s="77" t="s">
         <v>153</v>
       </c>
-      <c r="G36" s="79"/>
-      <c r="H36" s="79"/>
-      <c r="I36" s="79"/>
+      <c r="G36" s="78"/>
+      <c r="H36" s="78"/>
+      <c r="I36" s="78"/>
     </row>
     <row r="37" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A37" s="4" t="str">
@@ -22995,12 +22995,12 @@
         <v>1</v>
       </c>
       <c r="E43" s="36"/>
-      <c r="F43" s="78" t="s">
+      <c r="F43" s="77" t="s">
         <v>155</v>
       </c>
-      <c r="G43" s="79"/>
-      <c r="H43" s="79"/>
-      <c r="I43" s="79"/>
+      <c r="G43" s="78"/>
+      <c r="H43" s="78"/>
+      <c r="I43" s="78"/>
     </row>
     <row r="44" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A44" s="4" t="str">
@@ -23390,12 +23390,12 @@
         <v>1</v>
       </c>
       <c r="E50" s="36"/>
-      <c r="F50" s="78" t="s">
+      <c r="F50" s="77" t="s">
         <v>157</v>
       </c>
-      <c r="G50" s="79"/>
-      <c r="H50" s="79"/>
-      <c r="I50" s="79"/>
+      <c r="G50" s="78"/>
+      <c r="H50" s="78"/>
+      <c r="I50" s="78"/>
     </row>
     <row r="51" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A51" s="4" t="str">

</xml_diff>